<commit_message>
End of The Day 11/07/2026
</commit_message>
<xml_diff>
--- a/Flat/Data/utilities_history.xlsx
+++ b/Flat/Data/utilities_history.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J2"/>
+  <dimension ref="A1:J3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -528,6 +528,40 @@
         <v>6420.05</v>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>июнь 2026</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>1883.52</v>
+      </c>
+      <c r="C3" t="n">
+        <v>436</v>
+      </c>
+      <c r="D3" t="n">
+        <v>530.63</v>
+      </c>
+      <c r="E3" t="n">
+        <v>14.67</v>
+      </c>
+      <c r="F3" t="n">
+        <v>758.3</v>
+      </c>
+      <c r="G3" t="n">
+        <v>690</v>
+      </c>
+      <c r="H3" t="n">
+        <v>137.48</v>
+      </c>
+      <c r="I3" t="n">
+        <v>43.39</v>
+      </c>
+      <c r="J3" t="n">
+        <v>4043.32</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>